<commit_message>
fix extract sql file
</commit_message>
<xml_diff>
--- a/output_test/data_catalog.xlsx
+++ b/output_test/data_catalog.xlsx
@@ -612,7 +612,7 @@
       <c r="L2" s="3" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr"/>
@@ -652,7 +652,7 @@
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr"/>
@@ -692,7 +692,7 @@
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr"/>
@@ -723,7 +723,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="29" customWidth="1" min="13" max="13"/>
@@ -928,7 +928,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>don_vi_tinh IN (Vien, Vi, Hop, Chai</t>
+          <t>don_vi_tinh IN (Vien, Vi, Hop, Chai)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>

</xml_diff>